<commit_message>
Removed residency column from kyc import file (#1249)
</commit_message>
<xml_diff>
--- a/public/sample_uploads/investor_kycs.xlsx
+++ b/public/sample_uploads/investor_kycs.xlsx
@@ -207,8 +207,7 @@
             <family val="0"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">-Mandatory
--Please add custom fields for further bifurcations</t>
+          <t xml:space="preserve">-Optional</t>
         </r>
       </text>
     </comment>
@@ -323,34 +322,11 @@
             <family val="0"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">-Optional</t>
+          <t xml:space="preserve">-Mandatory</t>
         </r>
       </text>
     </comment>
     <comment ref="N1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="0"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">-Mandatory</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -374,7 +350,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -398,7 +374,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -422,6 +398,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="Q1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Author:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="0"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">-Mandatory for Angel Funds
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="R1" authorId="0">
       <text>
         <r>
@@ -446,31 +446,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="0"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">-Mandatory for Angel Funds
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -509,7 +485,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="62">
   <si>
     <t xml:space="preserve">Stakeholder</t>
   </si>
@@ -532,9 +508,6 @@
     <t xml:space="preserve">KYC Type *</t>
   </si>
   <si>
-    <t xml:space="preserve">Residency *</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bank Name</t>
   </si>
   <si>
@@ -589,9 +562,6 @@
     <t xml:space="preserve">Individual</t>
   </si>
   <si>
-    <t xml:space="preserve">Domestic</t>
-  </si>
-  <si>
     <t xml:space="preserve">HDFC</t>
   </si>
   <si>
@@ -632,9 +602,6 @@
   </si>
   <si>
     <t xml:space="preserve">D110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foreign</t>
   </si>
   <si>
     <t xml:space="preserve">BOB</t>
@@ -837,16 +804,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1120,7 +1083,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.56"/>
@@ -1130,355 +1093,335 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="21.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="19.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="12.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="8.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="8.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="18" style="1" width="11.92"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="22" style="1" width="8.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="8.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="22.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="17" style="1" width="11.92"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1022" min="21" style="1" width="8.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="10.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="4" t="n">
+        <v>27478</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>27478</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="n">
+        <v>50100000000</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="1" t="n">
-        <v>50100000000</v>
-      </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="S2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="7" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="S2" s="7" t="s">
+      <c r="T2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="T2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="U2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>15772</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="5" t="n">
-        <v>15772</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="G3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="1" t="n">
+        <v>50100000001</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="M3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="S3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="T3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>50100000001</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="R3" s="1" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="T3" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="U3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>33529</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>33529</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="J4" s="1" t="n">
+        <v>50100000002</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="M4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K4" s="1" t="n">
-        <v>50100000002</v>
-      </c>
-      <c r="L4" s="1" t="s">
+      <c r="Q4" s="1" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="S4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="U4" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" s="1" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T4" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="U4" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>36676</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>36676</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="J5" s="1" t="n">
+        <v>50100000003</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="M5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q5" s="1" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="R5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="S5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="T5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="U5" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>50100000003</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="R5" s="1" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="U5" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G1005" type="list">
       <formula1>"Individual,Non Individual"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="N2:P1005" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M2:O1005" type="list">
       <formula1>"Yes,No"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H1005" type="list">
-      <formula1>"Domestic,Foreign"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="Q2" r:id="rId2" display="signatory1@gmail.com,signatory2@gmail.com"/>
-    <hyperlink ref="Q3" r:id="rId3" display="signatory1@gmail.com,signatory2@gmail.com"/>
+    <hyperlink ref="P2" r:id="rId2" display="signatory1@gmail.com,signatory2@gmail.com"/>
+    <hyperlink ref="P3" r:id="rId3" display="signatory1@gmail.com,signatory2@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>